<commit_message>
add MLflow demo, update MLflow, add lakeFS, postgres, update docker compose in MLOps
</commit_message>
<xml_diff>
--- a/MLOps/MLflow/demo/train_test/runs_info.xlsx
+++ b/MLOps/MLflow/demo/train_test/runs_info.xlsx
@@ -461,174 +461,174 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>metrics.val_loss</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>metrics.val_MulticlassF1Score</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>metrics.system/gpu_0_memory_usage_percentage</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>metrics.system/disk_usage_megabytes</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>metrics.system/disk_usage_percentage</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>metrics.system/network_transmit_megabytes</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>metrics.system/gpu_0_power_usage_watts</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>metrics.system/network_receive_megabytes</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>metrics.train_MulticlassAccuracy</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>metrics.system/gpu_0_memory_usage_megabytes</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>metrics.system/gpu_0_utilization_percentage</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>metrics.system/system_memory_usage_percentage</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>metrics.train_MulticlassF1Score</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>metrics.system/system_memory_usage_megabytes</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>metrics.val_MulticlassAccuracy</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>metrics.train_loss</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>metrics.system/disk_available_megabytes</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>metrics.system/gpu_0_power_usage_percentage</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>metrics.system/cpu_utilization_percentage</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>metrics.system/system_memory_usage_percentage</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>metrics.train_MulticlassF1Score</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>metrics.system/disk_usage_megabytes</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>metrics.system/gpu_0_memory_usage_percentage</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>metrics.train_loss</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>metrics.train_MulticlassAccuracy</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>metrics.val_MulticlassF1Score</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>metrics.system/gpu_0_power_usage_percentage</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>metrics.system/gpu_0_power_usage_watts</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>metrics.system/network_transmit_megabytes</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>metrics.val_MulticlassAccuracy</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>metrics.system/gpu_0_memory_usage_megabytes</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>metrics.system/disk_usage_percentage</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>metrics.system/disk_available_megabytes</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>metrics.system/gpu_0_utilization_percentage</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>metrics.system/network_receive_megabytes</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>metrics.val_loss</t>
-        </is>
-      </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
+          <t>params. Metric 0</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>params.Batch size</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>params.Lr</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>params. Metric 1</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>params.Loss</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
           <t>params.Optimizer</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>params. Metric 0</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>params.Lr</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>params.Batch size</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>params.Epochs</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>params. Metric 1</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>params.Loss</t>
-        </is>
-      </c>
       <c r="AG1" s="1" t="inlineStr">
         <is>
+          <t>tags.mlflow.source.type</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>tags.mlflow.source.git.commit</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>tags.mlflow.log-model.history</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
           <t>tags.mlflow.source.name</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>tags.mlflow.user</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>tags.mlflow.runName</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>tags.mlflow.user</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>tags.mlflow.source.type</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>tags.mlflow.log-model.history</t>
-        </is>
-      </c>
-      <c r="AL1" s="1" t="inlineStr">
-        <is>
-          <t>tags.mlflow.source.git.commit</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>23c224087fad43448546fbeedc04ef47</t>
+          <t>31f2b68115e2414997945e93131b547c</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>701968018038163944</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -638,139 +638,139 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>mlflow-artifacts:/701968018038163944/23c224087fad43448546fbeedc04ef47/artifacts</t>
+          <t>mlflow-artifacts:/1/31f2b68115e2414997945e93131b547c/artifacts</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2024-12-06 13:01:47</t>
+          <t>2024-12-07 20:23:53</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2024-12-06 13:02:25</t>
+          <t>2024-12-07 20:40:15</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>14462.4</v>
+        <v>2.301549760601189</v>
       </c>
       <c r="H2" t="n">
-        <v>4.2</v>
+        <v>0.1091285720467567</v>
       </c>
       <c r="I2" t="n">
-        <v>21.6</v>
+        <v>4.7</v>
       </c>
       <c r="J2" t="n">
-        <v>0.9609853029251099</v>
+        <v>563089.3</v>
       </c>
       <c r="K2" t="n">
-        <v>556949.1</v>
+        <v>59</v>
       </c>
       <c r="L2" t="n">
-        <v>4.7</v>
+        <v>101.829346</v>
       </c>
       <c r="M2" t="n">
-        <v>0.2566874921321869</v>
+        <v>33.9</v>
       </c>
       <c r="N2" t="n">
-        <v>0.9609853029251099</v>
+        <v>96.94559800000025</v>
       </c>
       <c r="O2" t="n">
-        <v>0.9614914059638977</v>
+        <v>0.1093147024512291</v>
       </c>
       <c r="P2" t="n">
-        <v>27.8</v>
+        <v>801.3</v>
       </c>
       <c r="Q2" t="n">
-        <v>34.7</v>
+        <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>11.67677200000003</v>
+        <v>19.9</v>
       </c>
       <c r="S2" t="n">
-        <v>0.9614914059638977</v>
+        <v>0.1093147024512291</v>
       </c>
       <c r="T2" t="n">
-        <v>801.3</v>
+        <v>13374.4</v>
       </c>
       <c r="U2" t="n">
-        <v>58.3</v>
+        <v>0.1091285720467567</v>
       </c>
       <c r="V2" t="n">
-        <v>397748.1</v>
+        <v>2.306280374526978</v>
       </c>
       <c r="W2" t="n">
-        <v>3</v>
+        <v>391607.9</v>
       </c>
       <c r="X2" t="n">
-        <v>9.140529999999671</v>
+        <v>27.1</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.06411980722715513</v>
+        <v>4.1</v>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
+          <t>MulticlassAccuracy</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>0.9999999999999999</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>MulticlassF1Score</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>CrossEntropyLoss</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
           <t>SGD</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>MulticlassAccuracy</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>0.09999999999999999</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>128</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>MulticlassF1Score</t>
-        </is>
-      </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>CrossEntropyLoss</t>
-        </is>
-      </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>/home/trong/Downloads/Local/Source/Python/semester_9/AIP391/Video_anomaly_detection/MLOps/MLflow/demo/main.py</t>
+          <t>LOCAL</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>run 2</t>
+          <t>245450e4718602e614261c7e90c95dc2fc524a03</t>
         </is>
       </c>
       <c r="AI2" t="inlineStr">
         <is>
+          <t>[{"run_id": "31f2b68115e2414997945e93131b547c", "artifact_path": "model", "utc_time_created": "2024-12-07 13:40:12.251213", "model_uuid": "fb76f732a4af43f6a7bf82d3cdb461f4", "flavors": {"pytorch": {"model_data": "data", "pytorch_version": "2.5.0+cu124", "code": null}, "python_function": {"pickle_module_name": "mlflow.pytorch.pickle_module", "loader_module": "mlflow.pytorch", "python_version": "3.11.10", "data": "data", "env": {"conda": "conda.yaml", "virtualenv": "python_env.yaml"}}}}]</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>/home/trong/Downloads/Local/Source/Python/semester_9/AIP391/Video_anomaly_detection/MLOps/MLflow/demo/train_test/main.py</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
           <t>trong</t>
         </is>
       </c>
-      <c r="AJ2" t="inlineStr">
-        <is>
-          <t>LOCAL</t>
-        </is>
-      </c>
-      <c r="AK2" t="inlineStr">
-        <is>
-          <t>[{"run_id": "23c224087fad43448546fbeedc04ef47", "artifact_path": "model", "utc_time_created": "2024-12-06 06:02:23.015031", "model_uuid": "2ebc6dfb170c4715b9a87bbd6c630e79", "flavors": {"pytorch": {"model_data": "data", "pytorch_version": "2.5.0+cu124", "code": null}, "python_function": {"pickle_module_name": "mlflow.pytorch.pickle_module", "loader_module": "mlflow.pytorch", "python_version": "3.11.10", "data": "data", "env": {"conda": "conda.yaml", "virtualenv": "python_env.yaml"}}}}]</t>
-        </is>
-      </c>
       <c r="AL2" t="inlineStr">
         <is>
-          <t>cb28af176e95c6c4bc3b5cd59682ffa848159aaa</t>
+          <t>run 3</t>
         </is>
       </c>
     </row>

</xml_diff>